<commit_message>
new org_data format xdd
</commit_message>
<xml_diff>
--- a/org_templates/organization_card_example.xlsx
+++ b/org_templates/organization_card_example.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
   <si>
     <t xml:space="preserve">№ п/п</t>
   </si>
@@ -210,13 +210,22 @@
     <t xml:space="preserve">630099, Новосибирская область, г. Новосибирск, ул. Молодежная, д. 12, пом. 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Аудитор (должность, Ф.И.О. полностью)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Должность</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ф.И.О.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Эксперт по идентификации опасностей и оценке рисков</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Листикова Галина Михайловна</t>
+  </si>
+  <si>
     <t xml:space="preserve">Руководитель организации (должность, Ф.И.О. полностью)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Должность</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ф.И.О.</t>
   </si>
   <si>
     <t xml:space="preserve">Управляющий директор</t>
@@ -251,7 +260,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -329,22 +338,6 @@
       <sz val="12"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -410,16 +403,16 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -467,6 +460,10 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -475,15 +472,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -566,8 +563,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="42.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="61.29"/>
@@ -699,20 +696,20 @@
       <c r="A11" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="16" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="16" t="s">
+      <c r="B12" s="14"/>
+      <c r="C12" s="17" t="s">
         <v>19</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -726,21 +723,21 @@
       <c r="B13" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="16" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7"/>
       <c r="B14" s="8"/>
-      <c r="C14" s="16" t="s">
-        <v>19</v>
+      <c r="C14" s="18" t="s">
+        <v>22</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -748,42 +745,66 @@
         <v>12</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="16" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7"/>
       <c r="B16" s="8"/>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="17"/>
-      <c r="C17" s="3" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="C17" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="18" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="18"/>
+      <c r="D18" s="4" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="17"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="19"/>
+    </row>
+    <row r="21" customFormat="false" ht="42.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="18">
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
@@ -800,6 +821,8 @@
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="B15:B16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:B18"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>